<commit_message>
remove a URL de registro para bloquear bots
</commit_message>
<xml_diff>
--- a/Panilha_usuarios_controle.xlsx
+++ b/Panilha_usuarios_controle.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\PROJETOS\BOLAO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4051C4AD-CAD8-4691-A672-44981925E7FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{812F8BF4-D259-4B5D-BEA9-304A560002CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AE553B15-36E8-43BB-853A-88642CBD925A}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>Participante</t>
   </si>
@@ -50,9 +50,6 @@
     <t>SENHA</t>
   </si>
   <si>
-    <t>gustavolcbarbosa</t>
-  </si>
-  <si>
     <t>glcb2017</t>
   </si>
   <si>
@@ -66,6 +63,36 @@
   </si>
   <si>
     <t>lucas2017</t>
+  </si>
+  <si>
+    <t>Theolira</t>
+  </si>
+  <si>
+    <t>PIX</t>
+  </si>
+  <si>
+    <t>Theo Lira</t>
+  </si>
+  <si>
+    <t>gustavolopes</t>
+  </si>
+  <si>
+    <t>sim</t>
+  </si>
+  <si>
+    <t>não</t>
+  </si>
+  <si>
+    <t>vasco2026</t>
+  </si>
+  <si>
+    <t>Elaine de Abreu</t>
+  </si>
+  <si>
+    <t>ElainedeAbreu</t>
+  </si>
+  <si>
+    <t>flamengo26</t>
   </si>
 </sst>
 </file>
@@ -437,13 +464,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4555CD74-F6C1-496A-A5E3-689226333161}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -453,27 +480,64 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
         <v>8</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>